<commit_message>
fix: update ingredients in api route
</commit_message>
<xml_diff>
--- a/Piezas_a_contar.xlsx
+++ b/Piezas_a_contar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\Reportes-Cierres\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D71881DA-2278-4993-BDF2-DEC3C989057D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{182DB97E-2947-483B-93FA-BE2E6121A976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{2567D488-052E-4766-BA15-30F66857CA1B}"/>
   </bookViews>
@@ -988,7 +988,7 @@
       <c r="I6" s="5">
         <v>2</v>
       </c>
-      <c r="M6" s="6">
+      <c r="M6" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       <c r="J7" s="5">
         <v>1</v>
       </c>
-      <c r="M7" s="6">
+      <c r="M7" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       <c r="I8" s="5">
         <v>1</v>
       </c>
-      <c r="M8" s="6">
+      <c r="M8" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1063,7 +1063,7 @@
       <c r="J9" s="5">
         <v>2</v>
       </c>
-      <c r="M9" s="6">
+      <c r="M9" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
       <c r="I10" s="5">
         <v>1</v>
       </c>
-      <c r="M10" s="6">
+      <c r="M10" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1106,15 +1106,16 @@
       <c r="E11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="O11" s="6">
-        <v>1</v>
-      </c>
-      <c r="P11" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q11" s="6">
-        <v>1</v>
-      </c>
+      <c r="O11" s="5">
+        <v>1</v>
+      </c>
+      <c r="P11" s="5">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="5">
+        <v>1</v>
+      </c>
+      <c r="R11" s="5"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
@@ -1135,12 +1136,14 @@
       <c r="N12" s="6">
         <v>2</v>
       </c>
-      <c r="P12" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q12" s="6">
-        <v>1</v>
-      </c>
+      <c r="O12" s="5"/>
+      <c r="P12" s="5">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="5">
+        <v>1</v>
+      </c>
+      <c r="R12" s="5"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
@@ -1164,7 +1167,10 @@
       <c r="L13" s="5">
         <v>8</v>
       </c>
-      <c r="R13" s="6">
+      <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1190,6 +1196,10 @@
       <c r="L14" s="5">
         <v>1</v>
       </c>
+      <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="5"/>
+      <c r="R14" s="5"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
@@ -1207,6 +1217,10 @@
       <c r="E15" s="2" t="s">
         <v>74</v>
       </c>
+      <c r="O15" s="5"/>
+      <c r="P15" s="5"/>
+      <c r="Q15" s="5"/>
+      <c r="R15" s="5"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
@@ -1227,6 +1241,10 @@
       <c r="H16" s="5">
         <v>25</v>
       </c>
+      <c r="O16" s="5"/>
+      <c r="P16" s="5"/>
+      <c r="Q16" s="5"/>
+      <c r="R16" s="5"/>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
@@ -1247,6 +1265,10 @@
       <c r="H17" s="5">
         <v>25</v>
       </c>
+      <c r="O17" s="5"/>
+      <c r="P17" s="5"/>
+      <c r="Q17" s="5"/>
+      <c r="R17" s="5"/>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
@@ -1267,6 +1289,10 @@
       <c r="H18" s="5">
         <v>50</v>
       </c>
+      <c r="O18" s="5"/>
+      <c r="P18" s="5"/>
+      <c r="Q18" s="5"/>
+      <c r="R18" s="5"/>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
@@ -1287,6 +1313,10 @@
       <c r="H19" s="5">
         <v>50</v>
       </c>
+      <c r="O19" s="5"/>
+      <c r="P19" s="5"/>
+      <c r="Q19" s="5"/>
+      <c r="R19" s="5"/>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
@@ -1307,7 +1337,10 @@
       <c r="G20" s="5">
         <v>12</v>
       </c>
-      <c r="R20" s="6">
+      <c r="O20" s="5"/>
+      <c r="P20" s="5"/>
+      <c r="Q20" s="5"/>
+      <c r="R20" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1330,7 +1363,10 @@
       <c r="G21" s="5">
         <v>12</v>
       </c>
-      <c r="R21" s="6">
+      <c r="O21" s="5"/>
+      <c r="P21" s="5"/>
+      <c r="Q21" s="5"/>
+      <c r="R21" s="5">
         <v>1</v>
       </c>
     </row>

</xml_diff>